<commit_message>
Add personalized travel selection factors
</commit_message>
<xml_diff>
--- a/outputs/rmq-kkj-20260925/台中北九州_2026-09-25行程比較.xlsx
+++ b/outputs/rmq-kkj-20260925/台中北九州_2026-09-25行程比較.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9-25推薦" sheetId="1" r:id="R8bc0c31510c844a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行程比較" sheetId="2" r:id="R26e1ba06d07246a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐日明細" sheetId="3" r:id="Rb48076df69724eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通路價差" sheetId="4" r:id="R1e517892891a47ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="評分規則" sheetId="5" r:id="R68eb6de15e0040c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9-25推薦" sheetId="1" r:id="Rb3b180eed3724331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="行程比較" sheetId="2" r:id="R3f3f35256e56444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐日明細" sheetId="3" r:id="R2f516d9b2ea34039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通路價差" sheetId="4" r:id="R975ed5e489e9470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="評分規則" sheetId="5" r:id="R72f1dcb0439248e5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -255,7 +255,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="zinojeng" id="{D8ACCEB5-A77B-41CA-8CF0-814E10AE167B}"/>
+  <xltc:person displayName="zinojeng" id="{1580EBEC-5E8E-4A66-9841-D068511A3714}"/>
 </xltc:personList>
 </file>
 
@@ -582,32 +582,32 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="38" t="str">
-        <x:f>'行程比較'!C2</x:f>
-        <x:v>旅遊家旅行社</x:v>
+        <x:f>'行程比較'!C3</x:f>
+        <x:v>華府旅行社</x:v>
       </x:c>
       <x:c r="C5" s="39" t="str">
-        <x:f>'行程比較'!E2</x:f>
-        <x:v>九州神話秘境5日：高千穗、南阿蘇鐵道、柳川、糸島、雙溫泉</x:v>
+        <x:f>'行程比較'!E3</x:f>
+        <x:v>北九州山口5日：Safari Land、秋芳洞、琉璃光寺、元乃隅神社、角島</x:v>
       </x:c>
       <x:c r="D5" s="40" t="n">
-        <x:f>'行程比較'!F2</x:f>
-        <x:v>35900</x:v>
+        <x:f>'行程比較'!F3</x:f>
+        <x:v>43900</x:v>
       </x:c>
       <x:c r="E5" s="38" t="n">
-        <x:f>'行程比較'!N2</x:f>
+        <x:f>'行程比較'!N3</x:f>
         <x:v>80</x:v>
       </x:c>
       <x:c r="F5" s="41" t="str">
-        <x:f>"自由"&amp;'行程比較'!I2&amp;"日／自理"&amp;'行程比較'!J2&amp;"餐"</x:f>
+        <x:f>"自由"&amp;'行程比較'!I3&amp;"日／自理"&amp;'行程比較'!J3&amp;"餐"</x:f>
         <x:v>自由0日／自理1餐</x:v>
       </x:c>
       <x:c r="G5" s="41" t="str">
-        <x:f>"免稅"&amp;'行程比較'!K2&amp;"／商場"&amp;'行程比較'!L2&amp;"／見學"&amp;'行程比較'!M2</x:f>
+        <x:f>"免稅"&amp;'行程比較'!K3&amp;"／商場"&amp;'行程比較'!L3&amp;"／見學"&amp;'行程比較'!M3</x:f>
         <x:v>免稅1／商場1／見學0</x:v>
       </x:c>
       <x:c r="H5" s="41" t="str">
-        <x:f>'行程比較'!Q2</x:f>
-        <x:v>最符合偏好，建議優先詢問</x:v>
+        <x:f>'行程比較'!Q3</x:f>
+        <x:v>內容完整，但比旅遊家貴8,000元</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="52" customHeight="1">
@@ -615,32 +615,32 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="38" t="str">
-        <x:f>'行程比較'!C3</x:f>
-        <x:v>華府旅行社</x:v>
+        <x:f>'行程比較'!C4</x:f>
+        <x:v>山富旅遊</x:v>
       </x:c>
       <x:c r="C6" s="39" t="str">
-        <x:f>'行程比較'!E3</x:f>
-        <x:v>北九州山口5日：Safari Land、秋芳洞、琉璃光寺、元乃隅神社、角島</x:v>
+        <x:f>'行程比較'!E4</x:f>
+        <x:v>超值好運北九州鐵道5日：海景電車、賞豚、高千穗、熊本熊電鐵</x:v>
       </x:c>
       <x:c r="D6" s="40" t="n">
-        <x:f>'行程比較'!F3</x:f>
-        <x:v>43900</x:v>
+        <x:f>'行程比較'!F4</x:f>
+        <x:v>36900</x:v>
       </x:c>
       <x:c r="E6" s="38" t="n">
-        <x:f>'行程比較'!N3</x:f>
-        <x:v>80</x:v>
+        <x:f>'行程比較'!N4</x:f>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F6" s="41" t="str">
-        <x:f>"自由"&amp;'行程比較'!I3&amp;"日／自理"&amp;'行程比較'!J3&amp;"餐"</x:f>
+        <x:f>"自由"&amp;'行程比較'!I4&amp;"日／自理"&amp;'行程比較'!J4&amp;"餐"</x:f>
         <x:v>自由0日／自理1餐</x:v>
       </x:c>
       <x:c r="G6" s="41" t="str">
-        <x:f>"免稅"&amp;'行程比較'!K3&amp;"／商場"&amp;'行程比較'!L3&amp;"／見學"&amp;'行程比較'!M3</x:f>
-        <x:v>免稅1／商場1／見學0</x:v>
+        <x:f>"免稅"&amp;'行程比較'!K4&amp;"／商場"&amp;'行程比較'!L4&amp;"／見學"&amp;'行程比較'!M4</x:f>
+        <x:v>免稅1／商場2／見學1</x:v>
       </x:c>
       <x:c r="H6" s="41" t="str">
-        <x:f>'行程比較'!Q3</x:f>
-        <x:v>內容完整，但比旅遊家貴8,000元</x:v>
+        <x:f>'行程比較'!Q4</x:f>
+        <x:v>活動豐富，購物量中等</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="52" customHeight="1">
@@ -648,32 +648,32 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="38" t="str">
-        <x:f>'行程比較'!C4</x:f>
+        <x:f>'行程比較'!C5</x:f>
         <x:v>山富旅遊</x:v>
       </x:c>
       <x:c r="C7" s="39" t="str">
-        <x:f>'行程比較'!E4</x:f>
-        <x:v>超值好運北九州鐵道5日：海景電車、賞豚、高千穗、熊本熊電鐵</x:v>
+        <x:f>'行程比較'!E5</x:f>
+        <x:v>超值全覽北九州宮崎5日：由布院、日南海岸、鵜戶神宮、青井阿蘇神社</x:v>
       </x:c>
       <x:c r="D7" s="40" t="n">
-        <x:f>'行程比較'!F4</x:f>
+        <x:f>'行程比較'!F5</x:f>
         <x:v>36900</x:v>
       </x:c>
       <x:c r="E7" s="38" t="n">
-        <x:f>'行程比較'!N4</x:f>
+        <x:f>'行程比較'!N5</x:f>
         <x:v>72</x:v>
       </x:c>
       <x:c r="F7" s="41" t="str">
-        <x:f>"自由"&amp;'行程比較'!I4&amp;"日／自理"&amp;'行程比較'!J4&amp;"餐"</x:f>
+        <x:f>"自由"&amp;'行程比較'!I5&amp;"日／自理"&amp;'行程比較'!J5&amp;"餐"</x:f>
         <x:v>自由0日／自理1餐</x:v>
       </x:c>
       <x:c r="G7" s="41" t="str">
-        <x:f>"免稅"&amp;'行程比較'!K4&amp;"／商場"&amp;'行程比較'!L4&amp;"／見學"&amp;'行程比較'!M4</x:f>
-        <x:v>免稅1／商場2／見學1</x:v>
+        <x:f>"免稅"&amp;'行程比較'!K5&amp;"／商場"&amp;'行程比較'!L5&amp;"／見學"&amp;'行程比較'!M5</x:f>
+        <x:v>免稅1／商場1／見學2</x:v>
       </x:c>
       <x:c r="H7" s="41" t="str">
-        <x:f>'行程比較'!Q4</x:f>
-        <x:v>活動豐富，購物量中等</x:v>
+        <x:f>'行程比較'!Q5</x:f>
+        <x:v>無自由活動，購物略多</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52" customHeight="1">
@@ -681,32 +681,32 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="38" t="str">
-        <x:f>'行程比較'!C5</x:f>
-        <x:v>山富旅遊</x:v>
+        <x:f>'行程比較'!C2</x:f>
+        <x:v>旅遊家旅行社</x:v>
       </x:c>
       <x:c r="C8" s="39" t="str">
-        <x:f>'行程比較'!E5</x:f>
-        <x:v>超值全覽北九州宮崎5日：由布院、日南海岸、鵜戶神宮、青井阿蘇神社</x:v>
+        <x:f>'行程比較'!E2</x:f>
+        <x:v>九州神話秘境5日：高千穗、南阿蘇鐵道、柳川、糸島、雙溫泉</x:v>
       </x:c>
       <x:c r="D8" s="40" t="n">
-        <x:f>'行程比較'!F5</x:f>
-        <x:v>36900</x:v>
+        <x:f>'行程比較'!F2</x:f>
+        <x:v>35900</x:v>
       </x:c>
       <x:c r="E8" s="38" t="n">
-        <x:f>'行程比較'!N5</x:f>
-        <x:v>72</x:v>
+        <x:f>'行程比較'!N2</x:f>
+        <x:v>62.5</x:v>
       </x:c>
       <x:c r="F8" s="41" t="str">
-        <x:f>"自由"&amp;'行程比較'!I5&amp;"日／自理"&amp;'行程比較'!J5&amp;"餐"</x:f>
-        <x:v>自由0日／自理1餐</x:v>
+        <x:f>"自由"&amp;'行程比較'!I2&amp;"日／自理"&amp;'行程比較'!J2&amp;"餐"</x:f>
+        <x:v>自由0.5日／自理1餐</x:v>
       </x:c>
       <x:c r="G8" s="41" t="str">
-        <x:f>"免稅"&amp;'行程比較'!K5&amp;"／商場"&amp;'行程比較'!L5&amp;"／見學"&amp;'行程比較'!M5</x:f>
-        <x:v>免稅1／商場1／見學2</x:v>
+        <x:f>"免稅"&amp;'行程比較'!K2&amp;"／商場"&amp;'行程比較'!L2&amp;"／見學"&amp;'行程比較'!M2</x:f>
+        <x:v>免稅1／商場1／見學0</x:v>
       </x:c>
       <x:c r="H8" s="41" t="str">
-        <x:f>'行程比較'!Q5</x:f>
-        <x:v>無自由活動，購物略多</x:v>
+        <x:f>'行程比較'!Q2</x:f>
+        <x:v>特色餐與價格有優勢，但不再視為完全符合</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="52" customHeight="1">
@@ -816,13 +816,13 @@
         <x:v>快速判斷</x:v>
       </x:c>
       <x:c r="B13" s="42" t="str">
-        <x:v>旅遊家FUK05260925A</x:v>
+        <x:v>華府Safari CIKKJ260925C</x:v>
       </x:c>
       <x:c r="C13" s="42" t="str">
-        <x:v>比Safari便宜8,000</x:v>
+        <x:v>比旅遊家高8,000</x:v>
       </x:c>
       <x:c r="D13" s="42" t="str">
-        <x:v>動物園非遊樂園</x:v>
+        <x:v>動物園非機械遊樂園</x:v>
       </x:c>
       <x:c r="E13" s="42" t="str">
         <x:v>豪斯登堡／FIT自由行</x:v>
@@ -852,7 +852,7 @@
         <x:v>為什麼首選</x:v>
       </x:c>
       <x:c r="B15" s="41" t="str">
-        <x:v>旅遊家只有1餐自理，沒有自由活動；雖有免稅店與LaLaport，但集中在同一天，9/25售價35,900元。</x:v>
+        <x:v>華府Safari團沒有自由活動、只有1餐自理，購物集中同一天；若連自然動物園也不要，改選山富鐵道或宮崎團。</x:v>
       </x:c>
       <x:c r="C15" s="41"/>
       <x:c r="D15" s="41"/>
@@ -863,10 +863,10 @@
     </x:row>
     <x:row r="16" ht="44" customHeight="1">
       <x:c r="A16" s="44" t="str">
-        <x:v>替代選擇</x:v>
+        <x:v>重要修正</x:v>
       </x:c>
       <x:c r="B16" s="41" t="str">
-        <x:v>華府Safari團同樣只有1餐自理、沒有自由活動；適合能接受動物園且偏好山口自然景觀的人。</x:v>
+        <x:v>旅遊家第5天公開頁面載有福岡半日自由活動，且午餐說明與餐表矛盾，因此降為普通並建議書面確認。</x:v>
       </x:c>
       <x:c r="C16" s="41"/>
       <x:c r="D16" s="41"/>
@@ -981,7 +981,7 @@
         <x:v>T01</x:v>
       </x:c>
       <x:c r="B2" s="38" t="str">
-        <x:v>首選</x:v>
+        <x:v>普通</x:v>
       </x:c>
       <x:c r="C2" s="38" t="str">
         <x:v>旅遊家旅行社</x:v>
@@ -1002,7 +1002,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I2" s="38" t="n">
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="J2" s="38" t="n">
         <x:v>1</x:v>
@@ -1018,16 +1018,16 @@
       </x:c>
       <x:c r="N2" s="38" t="n">
         <x:f>IF(H2&gt;0,0,MAX(0,'評分規則'!$B$2-I2*'評分規則'!$B$3-J2*'評分規則'!$B$4-K2*'評分規則'!$B$5-L2*'評分規則'!$B$6-M2*'評分規則'!$B$7))</x:f>
-        <x:v>80</x:v>
+        <x:v>62.5</x:v>
       </x:c>
       <x:c r="O2" s="41" t="str">
-        <x:v>只有第4天晚餐自理；免稅店與LaLaport集中同一天。價格、餐食與景點密度最均衡。</x:v>
+        <x:v>第5天公開頁面載有福岡半日自由活動；第5天午餐說明與餐表互相矛盾，報名前需書面確認。</x:v>
       </x:c>
       <x:c r="P2" s="41" t="str">
         <x:v>https://b2b.travelerts.com.tw/EW/GO/GroupDetail.asp?prodCd=FUK05260925A</x:v>
       </x:c>
       <x:c r="Q2" s="41" t="str">
-        <x:v>最符合偏好，建議優先詢問</x:v>
+        <x:v>特色餐與價格有優勢，但不再視為完全符合</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
@@ -1479,7 +1479,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra31db10a8e734807"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dda80f10e3f4ca5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1630,18 +1630,20 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="41" t="str">
-        <x:v>糸島夫婦岩→一蘭之森→機場</x:v>
+        <x:v>福岡半日自由活動→糸島→一蘭之森→機場</x:v>
       </x:c>
       <x:c r="D6" s="42" t="str">
         <x:v>飯店</x:v>
       </x:c>
       <x:c r="E6" s="42" t="str">
-        <x:v>一蘭拉麵</x:v>
+        <x:v>頁面說明矛盾，需確認</x:v>
       </x:c>
       <x:c r="F6" s="42" t="str">
         <x:v>機上餐</x:v>
       </x:c>
-      <x:c r="G6" s="41" t="str"/>
+      <x:c r="G6" s="41" t="str">
+        <x:v>半日自由；午餐需確認</x:v>
+      </x:c>
       <x:c r="H6" s="41" t="str">
         <x:v>https://b2b.travelerts.com.tw/EW/GO/GroupDetail.asp?prodCd=FUK05260925A</x:v>
       </x:c>
@@ -2657,7 +2659,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bb84e0969564c91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66ecd58bf91949dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2895,7 +2897,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d1b229a85254ee4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra36fb77c61834429"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>